<commit_message>
Observer extraction, refreshed Trektellen exports (15 Oct 2026), audit and docs updates
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/raw/trektellen/Trektellen_headerdata_2422_2023.xlsx
+++ b/raw/trektellen/Trektellen_headerdata_2422_2023.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="848">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="849">
   <si>
     <t>id</t>
   </si>
@@ -2363,7 +2363,7 @@
     <t>2023-11-11 07:40:00</t>
   </si>
   <si>
-    <t>2023-11-11 19:14:00</t>
+    <t>2023-11-11 17:15:00</t>
   </si>
   <si>
     <t>Dominique Maire, Pascal Charrière 7h30/17h15,Raymond Bedouet 10h45/12h15, Andrée Tieffenbach 11h/15h40, Lutz Lucker et Sylvie Freymond 12h25/17h, Isabelle et Roger Cattin Gasser 13h/17h15</t>
@@ -2373,6 +2373,9 @@
   </si>
   <si>
     <t>2023-12-07 17:29:07.36437</t>
+  </si>
+  <si>
+    <t>2026-10-14 17:38:24.600072</t>
   </si>
   <si>
     <t>2023-11-12 07:19:00</t>
@@ -9189,7 +9192,10 @@
         <v>37</v>
       </c>
       <c r="AC122" t="s">
-        <v>785</v>
+        <v>786</v>
+      </c>
+      <c r="AD122" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="123" spans="1:30">
@@ -9215,25 +9221,25 @@
         <v>2023</v>
       </c>
       <c r="H123" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="I123" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="K123" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="Y123" t="s">
         <v>34</v>
       </c>
       <c r="AA123" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="AB123" t="s">
         <v>37</v>
       </c>
       <c r="AC123" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="AD123" t="s">
         <v>37</v>
@@ -9262,28 +9268,28 @@
         <v>2023</v>
       </c>
       <c r="H124" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="I124" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="J124" t="s">
         <v>651</v>
       </c>
       <c r="K124" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="Y124" t="s">
         <v>34</v>
       </c>
       <c r="AA124" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="AB124" t="s">
         <v>37</v>
       </c>
       <c r="AC124" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="AD124" t="s">
         <v>37</v>
@@ -9312,28 +9318,28 @@
         <v>2023</v>
       </c>
       <c r="H125" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="I125" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="J125" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="K125" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="Y125" t="s">
         <v>34</v>
       </c>
       <c r="AA125" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="AB125" t="s">
         <v>37</v>
       </c>
       <c r="AC125" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="AD125" t="s">
         <v>37</v>
@@ -9362,28 +9368,28 @@
         <v>2023</v>
       </c>
       <c r="H126" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="I126" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="J126" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="K126" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="Y126" t="s">
         <v>34</v>
       </c>
       <c r="AA126" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="AB126" t="s">
         <v>37</v>
       </c>
       <c r="AC126" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="AD126" t="s">
         <v>37</v>
@@ -9412,28 +9418,28 @@
         <v>2023</v>
       </c>
       <c r="H127" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="I127" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="J127" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="K127" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="Y127" t="s">
         <v>34</v>
       </c>
       <c r="AA127" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="AB127" t="s">
         <v>37</v>
       </c>
       <c r="AC127" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="AD127" t="s">
         <v>37</v>
@@ -9462,28 +9468,28 @@
         <v>2023</v>
       </c>
       <c r="H128" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="I128" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="J128" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="K128" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="Y128" t="s">
         <v>34</v>
       </c>
       <c r="AA128" t="s">
-        <v>818</v>
+        <v>819</v>
       </c>
       <c r="AB128" t="s">
         <v>37</v>
       </c>
       <c r="AC128" t="s">
-        <v>819</v>
+        <v>820</v>
       </c>
       <c r="AD128" t="s">
         <v>37</v>
@@ -9512,28 +9518,28 @@
         <v>2023</v>
       </c>
       <c r="H129" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="I129" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="J129" t="s">
-        <v>822</v>
+        <v>823</v>
       </c>
       <c r="K129" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="Y129" t="s">
         <v>34</v>
       </c>
       <c r="AA129" t="s">
-        <v>824</v>
+        <v>825</v>
       </c>
       <c r="AB129" t="s">
         <v>37</v>
       </c>
       <c r="AC129" t="s">
-        <v>825</v>
+        <v>826</v>
       </c>
       <c r="AD129" t="s">
         <v>37</v>
@@ -9562,25 +9568,25 @@
         <v>2023</v>
       </c>
       <c r="H130" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="I130" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="J130" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="Y130" t="s">
         <v>34</v>
       </c>
       <c r="AA130" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="AB130" t="s">
         <v>37</v>
       </c>
       <c r="AC130" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="AD130" t="s">
         <v>37</v>
@@ -9609,25 +9615,25 @@
         <v>2023</v>
       </c>
       <c r="H131" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="I131" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="J131" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="Y131" t="s">
         <v>34</v>
       </c>
       <c r="AA131" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="AB131" t="s">
         <v>37</v>
       </c>
       <c r="AC131" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="AD131" t="s">
         <v>37</v>
@@ -9656,16 +9662,16 @@
         <v>2023</v>
       </c>
       <c r="H132" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="I132" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="J132" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="K132" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="N132" t="s">
         <v>665</v>
@@ -9677,13 +9683,13 @@
         <v>34</v>
       </c>
       <c r="AA132" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="AB132" t="s">
         <v>37</v>
       </c>
       <c r="AC132" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="AD132" t="s">
         <v>37</v>
@@ -9712,16 +9718,16 @@
         <v>2023</v>
       </c>
       <c r="H133" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="I133" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="J133" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="K133" t="s">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="N133" t="s">
         <v>493</v>
@@ -9733,13 +9739,13 @@
         <v>34</v>
       </c>
       <c r="AA133" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="AB133" t="s">
         <v>37</v>
       </c>
       <c r="AC133" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="AD133" t="s">
         <v>37</v>

</xml_diff>